<commit_message>
grok(yassir): 4-market economics cascade + growth_case splice (deck gate)
Preflight country-reference (MA/TN/DZ/SN, CAPEX $600K). Full cascade
aggregate→growth→splice over Morocco/Tunisia/Algeria/Senegal. Hub floor
34 boats / $10.8M rev / $115.8M pool replaces stale 43-boat / $111M splice
in both data-clean and partner-pitch yassir.json. Sidecar + local sheet
built; Drive publish pending OAuth tokens.
</commit_message>
<xml_diff>
--- a/finance/_refresh_yassir.xlsx
+++ b/finance/_refresh_yassir.xlsx
@@ -44,9 +44,9 @@
     <definedName name="scenario">'Assumptions'!$B$38</definedName>
     <definedName name="load_sel">'Assumptions'!$B$39</definedName>
     <definedName name="revleg_sel">'Assumptions'!$B$40</definedName>
-    <definedName name="country_opex">'Country opex'!$A$4:$G$6</definedName>
-    <definedName name="som_floor_fleet">'Corridor economics'!$D$28</definedName>
-    <definedName name="som_floor_rev">'Corridor economics'!$E$28</definedName>
+    <definedName name="country_opex">'Country opex'!$A$4:$G$7</definedName>
+    <definedName name="som_floor_fleet">'Corridor economics'!$D$33</definedName>
+    <definedName name="som_floor_rev">'Corridor economics'!$E$33</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1813,7 +1813,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1938,28 +1938,58 @@
     <row r="6">
       <c r="A6" s="25" t="inlineStr">
         <is>
-          <t>Tunisia</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="B6" s="26" t="n">
-        <v>14000</v>
+        <v>12000</v>
       </c>
       <c r="C6" s="27" t="n">
-        <v>0.1</v>
+        <v>0.18</v>
       </c>
       <c r="D6" s="19" t="n">
-        <v>0.45</v>
+        <v>0.55</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>9000</v>
+        <v>8000</v>
       </c>
       <c r="F6" s="19" t="n">
-        <v>0.35</v>
+        <v>0.32</v>
       </c>
       <c r="G6" s="26" t="n">
         <v>600000</v>
       </c>
       <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>Modeled from national maritime-wage / cost-of-living index vs SG anchor | Modeled from national commercial electricity tariff avg | Modeled berth/marina overhead vs SG anchor by cost index | CAPEX LB-243 US/EU=$900K else $600K</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="25" t="inlineStr">
+        <is>
+          <t>Tunisia</t>
+        </is>
+      </c>
+      <c r="B7" s="26" t="n">
+        <v>14000</v>
+      </c>
+      <c r="C7" s="27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D7" s="19" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E7" s="26" t="n">
+        <v>9000</v>
+      </c>
+      <c r="F7" s="19" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G7" s="26" t="n">
+        <v>600000</v>
+      </c>
+      <c r="H7" s="14" t="inlineStr">
         <is>
           <t>Modeled from national maritime-wage / cost-of-living index vs SG anchor | Modeled from national commercial electricity tariff avg | Modeled berth/marina overhead vs SG anchor by cost index | CAPEX LB-243 US/EU=$900K else $600K</t>
         </is>
@@ -1979,7 +2009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY33"/>
+  <dimension ref="A1:AY40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2316,7 +2346,7 @@
     <row r="4">
       <c r="A4" s="29" t="inlineStr">
         <is>
-          <t>Yassir Algeria</t>
+          <t>Yassir</t>
         </is>
       </c>
       <c r="B4" s="29" t="inlineStr">
@@ -2326,15 +2356,13 @@
       </c>
       <c r="C4" s="30" t="inlineStr">
         <is>
-          <t>La Pêcherie / Port d'Alger → El Djamila / Aïn Bénian</t>
+          <t>Port of Annaba (Môle Cigogne / Quai Nord) → Annaba Corniche — Plage Rizi Amor / Saint-Cloud</t>
         </is>
       </c>
       <c r="D4" s="31" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="E4" s="26" t="n">
-        <v>18</v>
-      </c>
+        <v>2.1</v>
+      </c>
+      <c r="E4" s="26" t="n"/>
       <c r="F4" s="32" t="n"/>
       <c r="G4" s="32" t="n"/>
       <c r="H4" s="19" t="n">
@@ -2436,9 +2464,7 @@
         <f>((D4*O4/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D4*O4*VLOOKUP(B4,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG4" s="31" t="n">
-        <v>170280</v>
-      </c>
+      <c r="AG4" s="31" t="n"/>
       <c r="AH4" s="32" t="n"/>
       <c r="AI4" s="32" t="n"/>
       <c r="AJ4" s="39" t="n">
@@ -2467,7 +2493,7 @@
       <c r="AP4" s="40" t="n"/>
       <c r="AQ4" s="32" t="inlineStr">
         <is>
-          <t>Grounded</t>
+          <t>Estimated</t>
         </is>
       </c>
       <c r="AR4" s="41" t="n"/>
@@ -2485,31 +2511,27 @@
         <f>IF(((S4*pax_cap*load_full*ROUND(K4*L4*revleg_full,0))-(((battery/range_nm)*D4*ROUND(K4*L4*revleg_full,0)*VLOOKUP(B4,country_opex,3,FALSE))+V4+W4+X4+Y4+Z4))&lt;=0,"",VLOOKUP(B4,country_opex,7,FALSE)/((S4*pax_cap*load_full*ROUND(K4*L4*revleg_full,0))-(((battery/range_nm)*D4*ROUND(K4*L4*revleg_full,0)*VLOOKUP(B4,country_opex,3,FALSE))+V4+W4+X4+Y4+Z4)))</f>
         <v/>
       </c>
-      <c r="AX4" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[LB-255 PREMIUM RE-FARE: subsidized comparable $3.7 lifted to premium on-demand floor $18.0] </t>
-        </is>
-      </c>
+      <c r="AX4" s="44" t="n"/>
       <c r="AY4" s="44" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="29" t="inlineStr">
         <is>
-          <t>Yassir Morocco</t>
+          <t>Yassir</t>
         </is>
       </c>
       <c r="B5" s="29" t="inlineStr">
         <is>
-          <t>Morocco</t>
+          <t>Algeria</t>
         </is>
       </c>
       <c r="C5" s="30" t="inlineStr">
         <is>
-          <t>Rabat → Sale</t>
+          <t>Gare Maritime / Port d'Oran → Ain El Turck / Kristel waterfront</t>
         </is>
       </c>
       <c r="D5" s="31" t="n">
-        <v>0.5</v>
+        <v>2.3</v>
       </c>
       <c r="E5" s="26" t="n"/>
       <c r="F5" s="32" t="n"/>
@@ -2666,23 +2688,25 @@
     <row r="6">
       <c r="A6" s="29" t="inlineStr">
         <is>
-          <t>Yassir Morocco</t>
+          <t>Yassir</t>
         </is>
       </c>
       <c r="B6" s="29" t="inlineStr">
         <is>
-          <t>Morocco</t>
+          <t>Algeria</t>
         </is>
       </c>
       <c r="C6" s="30" t="inlineStr">
         <is>
-          <t>Rabat → Sale</t>
+          <t>La Pêcherie / Port d'Alger → El Djamila / Aïn Bénian</t>
         </is>
       </c>
       <c r="D6" s="31" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E6" s="26" t="n"/>
+        <v>8.5</v>
+      </c>
+      <c r="E6" s="26" t="n">
+        <v>18</v>
+      </c>
       <c r="F6" s="32" t="n"/>
       <c r="G6" s="32" t="n"/>
       <c r="H6" s="19" t="n">
@@ -2697,7 +2721,7 @@
         <v/>
       </c>
       <c r="K6" s="34">
-        <f>MIN(24,FLOOR(60*service_hr/J6,1))</f>
+        <f>MIN(15,FLOOR(60*service_hr/J6,1))</f>
         <v/>
       </c>
       <c r="L6" s="34">
@@ -2784,7 +2808,9 @@
         <f>((D6*O6/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D6*O6*VLOOKUP(B6,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG6" s="31" t="n"/>
+      <c r="AG6" s="31" t="n">
+        <v>170280</v>
+      </c>
       <c r="AH6" s="32" t="n"/>
       <c r="AI6" s="32" t="n"/>
       <c r="AJ6" s="39" t="n">
@@ -2813,7 +2839,7 @@
       <c r="AP6" s="40" t="n"/>
       <c r="AQ6" s="32" t="inlineStr">
         <is>
-          <t>Estimated</t>
+          <t>Grounded</t>
         </is>
       </c>
       <c r="AR6" s="41" t="n"/>
@@ -2831,41 +2857,35 @@
         <f>IF(((S6*pax_cap*load_full*ROUND(K6*L6*revleg_full,0))-(((battery/range_nm)*D6*ROUND(K6*L6*revleg_full,0)*VLOOKUP(B6,country_opex,3,FALSE))+V6+W6+X6+Y6+Z6))&lt;=0,"",VLOOKUP(B6,country_opex,7,FALSE)/((S6*pax_cap*load_full*ROUND(K6*L6*revleg_full,0))-(((battery/range_nm)*D6*ROUND(K6*L6*revleg_full,0)*VLOOKUP(B6,country_opex,3,FALSE))+V6+W6+X6+Y6+Z6)))</f>
         <v/>
       </c>
-      <c r="AX6" s="44" t="n"/>
+      <c r="AX6" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[LB-255 PREMIUM RE-FARE: subsidized comparable $3.7 lifted to premium on-demand floor $18.0] </t>
+        </is>
+      </c>
       <c r="AY6" s="44" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="29" t="inlineStr">
         <is>
-          <t>Yassir Morocco</t>
+          <t>Yassir</t>
         </is>
       </c>
       <c r="B7" s="29" t="inlineStr">
         <is>
-          <t>Morocco</t>
+          <t>Algeria</t>
         </is>
       </c>
       <c r="C7" s="30" t="inlineStr">
         <is>
-          <t>Tangier Marina Bay → Tarifa (cross-strait excluded)</t>
+          <t>La Pêcherie / Port d'Alger / Gare Maritime → Tamentfoust (east bay harbour)</t>
         </is>
       </c>
       <c r="D7" s="31" t="n">
-        <v>8</v>
-      </c>
-      <c r="E7" s="26" t="n">
-        <v>43.5</v>
-      </c>
-      <c r="F7" s="32" t="inlineStr">
-        <is>
-          <t>T2</t>
-        </is>
-      </c>
-      <c r="G7" s="32" t="inlineStr">
-        <is>
-          <t>med</t>
-        </is>
-      </c>
+        <v>10.3</v>
+      </c>
+      <c r="E7" s="26" t="n"/>
+      <c r="F7" s="32" t="n"/>
+      <c r="G7" s="32" t="n"/>
       <c r="H7" s="19" t="n">
         <v>1</v>
       </c>
@@ -2965,9 +2985,7 @@
         <f>((D7*O7/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D7*O7*VLOOKUP(B7,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG7" s="31" t="n">
-        <v>760778</v>
-      </c>
+      <c r="AG7" s="31" t="n"/>
       <c r="AH7" s="32" t="n"/>
       <c r="AI7" s="32" t="n"/>
       <c r="AJ7" s="39" t="n">
@@ -2996,7 +3014,7 @@
       <c r="AP7" s="40" t="n"/>
       <c r="AQ7" s="32" t="inlineStr">
         <is>
-          <t>Grounded</t>
+          <t>Estimated</t>
         </is>
       </c>
       <c r="AR7" s="41" t="n"/>
@@ -3014,31 +3032,27 @@
         <f>IF(((S7*pax_cap*load_full*ROUND(K7*L7*revleg_full,0))-(((battery/range_nm)*D7*ROUND(K7*L7*revleg_full,0)*VLOOKUP(B7,country_opex,3,FALSE))+V7+W7+X7+Y7+Z7))&lt;=0,"",VLOOKUP(B7,country_opex,7,FALSE)/((S7*pax_cap*load_full*ROUND(K7*L7*revleg_full,0))-(((battery/range_nm)*D7*ROUND(K7*L7*revleg_full,0)*VLOOKUP(B7,country_opex,3,FALSE))+V7+W7+X7+Y7+Z7)))</f>
         <v/>
       </c>
-      <c r="AX7" s="44" t="inlineStr">
-        <is>
-          <t>PREMIUM tier: standard adult FOOT-PASSENGER one-way fast-ferry fare Tarifa&lt;-&gt;Tangier Ville ~EUR 40.25 (traveller-reported foot fare) x 1.08 = ~$43.5; DirectFerries lists 'from $46'. THIS is the Navier-modeled per-seat tier.</t>
-        </is>
-      </c>
+      <c r="AX7" s="44" t="n"/>
       <c r="AY7" s="44" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="29" t="inlineStr">
         <is>
-          <t>Yassir Morocco</t>
+          <t>Yassir</t>
         </is>
       </c>
       <c r="B8" s="29" t="inlineStr">
         <is>
-          <t>Morocco</t>
+          <t>Algeria</t>
         </is>
       </c>
       <c r="C8" s="30" t="inlineStr">
         <is>
-          <t>Agadir Marina → Taghazout</t>
+          <t>Port de Sidi Fredj (marina) → El Djamila / Aïn Bénian</t>
         </is>
       </c>
       <c r="D8" s="31" t="n">
-        <v>9</v>
+        <v>13.8</v>
       </c>
       <c r="E8" s="26" t="n"/>
       <c r="F8" s="32" t="n"/>
@@ -3142,9 +3156,7 @@
         <f>((D8*O8/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D8*O8*VLOOKUP(B8,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG8" s="31" t="n">
-        <v>77500</v>
-      </c>
+      <c r="AG8" s="31" t="n"/>
       <c r="AH8" s="32" t="n"/>
       <c r="AI8" s="32" t="n"/>
       <c r="AJ8" s="39" t="n">
@@ -3197,7 +3209,7 @@
     <row r="9">
       <c r="A9" s="29" t="inlineStr">
         <is>
-          <t>Yassir Morocco</t>
+          <t>Yassir</t>
         </is>
       </c>
       <c r="B9" s="29" t="inlineStr">
@@ -3207,11 +3219,11 @@
       </c>
       <c r="C9" s="30" t="inlineStr">
         <is>
-          <t>Casablanca → Mohammedia</t>
+          <t>Rabat → Sale</t>
         </is>
       </c>
       <c r="D9" s="31" t="n">
-        <v>13</v>
+        <v>0.5</v>
       </c>
       <c r="E9" s="26" t="n"/>
       <c r="F9" s="32" t="n"/>
@@ -3228,7 +3240,7 @@
         <v/>
       </c>
       <c r="K9" s="34">
-        <f>MIN(24,FLOOR(60*service_hr/J9,1))</f>
+        <f>MIN(15,FLOOR(60*service_hr/J9,1))</f>
         <v/>
       </c>
       <c r="L9" s="34">
@@ -3368,7 +3380,7 @@
     <row r="10">
       <c r="A10" s="29" t="inlineStr">
         <is>
-          <t>Yassir Morocco</t>
+          <t>Yassir</t>
         </is>
       </c>
       <c r="B10" s="29" t="inlineStr">
@@ -3378,25 +3390,15 @@
       </c>
       <c r="C10" s="30" t="inlineStr">
         <is>
-          <t>Tanger Med (Ksar el Majaz) → Algeciras (Spain)</t>
+          <t>Rabat → Sale</t>
         </is>
       </c>
       <c r="D10" s="31" t="n">
-        <v>13</v>
-      </c>
-      <c r="E10" s="26" t="n">
-        <v>38</v>
-      </c>
-      <c r="F10" s="32" t="inlineStr">
-        <is>
-          <t>T2</t>
-        </is>
-      </c>
-      <c r="G10" s="32" t="inlineStr">
-        <is>
-          <t>med</t>
-        </is>
-      </c>
+        <v>0.5</v>
+      </c>
+      <c r="E10" s="26" t="n"/>
+      <c r="F10" s="32" t="n"/>
+      <c r="G10" s="32" t="n"/>
       <c r="H10" s="19" t="n">
         <v>1</v>
       </c>
@@ -3409,7 +3411,7 @@
         <v/>
       </c>
       <c r="K10" s="34">
-        <f>MIN(15,FLOOR(60*service_hr/J10,1))</f>
+        <f>MIN(24,FLOOR(60*service_hr/J10,1))</f>
         <v/>
       </c>
       <c r="L10" s="34">
@@ -3496,9 +3498,7 @@
         <f>((D10*O10/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D10*O10*VLOOKUP(B10,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG10" s="31" t="n">
-        <v>1610211</v>
-      </c>
+      <c r="AG10" s="31" t="n"/>
       <c r="AH10" s="32" t="n"/>
       <c r="AI10" s="32" t="n"/>
       <c r="AJ10" s="39" t="n">
@@ -3527,7 +3527,7 @@
       <c r="AP10" s="40" t="n"/>
       <c r="AQ10" s="32" t="inlineStr">
         <is>
-          <t>Grounded</t>
+          <t>Estimated</t>
         </is>
       </c>
       <c r="AR10" s="41" t="n"/>
@@ -3545,17 +3545,13 @@
         <f>IF(((S10*pax_cap*load_full*ROUND(K10*L10*revleg_full,0))-(((battery/range_nm)*D10*ROUND(K10*L10*revleg_full,0)*VLOOKUP(B10,country_opex,3,FALSE))+V10+W10+X10+Y10+Z10))&lt;=0,"",VLOOKUP(B10,country_opex,7,FALSE)/((S10*pax_cap*load_full*ROUND(K10*L10*revleg_full,0))-(((battery/range_nm)*D10*ROUND(K10*L10*revleg_full,0)*VLOOKUP(B10,country_opex,3,FALSE))+V10+W10+X10+Y10+Z10)))</f>
         <v/>
       </c>
-      <c r="AX10" s="44" t="inlineStr">
-        <is>
-          <t>PREMIUM tier: standard adult FOOT-PASSENGER one-way Tanger Med&lt;-&gt;Algeciras ~EUR 35 x 1.08 = ~$38 (Strait fast-ferry foot fares cluster EUR 30-40).</t>
-        </is>
-      </c>
+      <c r="AX10" s="44" t="n"/>
       <c r="AY10" s="44" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="29" t="inlineStr">
         <is>
-          <t>Yassir Morocco</t>
+          <t>Yassir</t>
         </is>
       </c>
       <c r="B11" s="29" t="inlineStr">
@@ -3565,15 +3561,25 @@
       </c>
       <c r="C11" s="30" t="inlineStr">
         <is>
-          <t>Al Hoceima → Cala Iris</t>
+          <t>Tangier Marina Bay → Tarifa (cross-strait excluded)</t>
         </is>
       </c>
       <c r="D11" s="31" t="n">
-        <v>16</v>
-      </c>
-      <c r="E11" s="26" t="n"/>
-      <c r="F11" s="32" t="n"/>
-      <c r="G11" s="32" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="E11" s="26" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="F11" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G11" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
       <c r="H11" s="19" t="n">
         <v>1</v>
       </c>
@@ -3586,7 +3592,7 @@
         <v/>
       </c>
       <c r="K11" s="34">
-        <f>MIN(24,FLOOR(60*service_hr/J11,1))</f>
+        <f>MIN(15,FLOOR(60*service_hr/J11,1))</f>
         <v/>
       </c>
       <c r="L11" s="34">
@@ -3673,7 +3679,9 @@
         <f>((D11*O11/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D11*O11*VLOOKUP(B11,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG11" s="31" t="n"/>
+      <c r="AG11" s="31" t="n">
+        <v>760778</v>
+      </c>
       <c r="AH11" s="32" t="n"/>
       <c r="AI11" s="32" t="n"/>
       <c r="AJ11" s="39" t="n">
@@ -3702,7 +3710,7 @@
       <c r="AP11" s="40" t="n"/>
       <c r="AQ11" s="32" t="inlineStr">
         <is>
-          <t>Estimated</t>
+          <t>Grounded</t>
         </is>
       </c>
       <c r="AR11" s="41" t="n"/>
@@ -3720,13 +3728,17 @@
         <f>IF(((S11*pax_cap*load_full*ROUND(K11*L11*revleg_full,0))-(((battery/range_nm)*D11*ROUND(K11*L11*revleg_full,0)*VLOOKUP(B11,country_opex,3,FALSE))+V11+W11+X11+Y11+Z11))&lt;=0,"",VLOOKUP(B11,country_opex,7,FALSE)/((S11*pax_cap*load_full*ROUND(K11*L11*revleg_full,0))-(((battery/range_nm)*D11*ROUND(K11*L11*revleg_full,0)*VLOOKUP(B11,country_opex,3,FALSE))+V11+W11+X11+Y11+Z11)))</f>
         <v/>
       </c>
-      <c r="AX11" s="44" t="n"/>
+      <c r="AX11" s="44" t="inlineStr">
+        <is>
+          <t>PREMIUM tier: standard adult FOOT-PASSENGER one-way fast-ferry fare Tarifa&lt;-&gt;Tangier Ville ~EUR 40.25 (traveller-reported foot fare) x 1.08 = ~$43.5; DirectFerries lists 'from $46'. THIS is the Navier-modeled per-seat tier.</t>
+        </is>
+      </c>
       <c r="AY11" s="44" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="29" t="inlineStr">
         <is>
-          <t>Yassir Morocco</t>
+          <t>Yassir</t>
         </is>
       </c>
       <c r="B12" s="29" t="inlineStr">
@@ -3736,25 +3748,15 @@
       </c>
       <c r="C12" s="30" t="inlineStr">
         <is>
-          <t>Tanger Med → Ceuta (Spanish enclave)</t>
+          <t>Agadir Marina → Taghazout</t>
         </is>
       </c>
       <c r="D12" s="31" t="n">
-        <v>22</v>
-      </c>
-      <c r="E12" s="26" t="n">
-        <v>36</v>
-      </c>
-      <c r="F12" s="32" t="inlineStr">
-        <is>
-          <t>T2</t>
-        </is>
-      </c>
-      <c r="G12" s="32" t="inlineStr">
-        <is>
-          <t>med</t>
-        </is>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="E12" s="26" t="n"/>
+      <c r="F12" s="32" t="n"/>
+      <c r="G12" s="32" t="n"/>
       <c r="H12" s="19" t="n">
         <v>1</v>
       </c>
@@ -3854,7 +3856,9 @@
         <f>((D12*O12/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D12*O12*VLOOKUP(B12,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG12" s="31" t="n"/>
+      <c r="AG12" s="31" t="n">
+        <v>77500</v>
+      </c>
       <c r="AH12" s="32" t="n"/>
       <c r="AI12" s="32" t="n"/>
       <c r="AJ12" s="39" t="n">
@@ -3883,7 +3887,7 @@
       <c r="AP12" s="40" t="n"/>
       <c r="AQ12" s="32" t="inlineStr">
         <is>
-          <t>Estimated</t>
+          <t>Grounded</t>
         </is>
       </c>
       <c r="AR12" s="41" t="n"/>
@@ -3901,17 +3905,13 @@
         <f>IF(((S12*pax_cap*load_full*ROUND(K12*L12*revleg_full,0))-(((battery/range_nm)*D12*ROUND(K12*L12*revleg_full,0)*VLOOKUP(B12,country_opex,3,FALSE))+V12+W12+X12+Y12+Z12))&lt;=0,"",VLOOKUP(B12,country_opex,7,FALSE)/((S12*pax_cap*load_full*ROUND(K12*L12*revleg_full,0))-(((battery/range_nm)*D12*ROUND(K12*L12*revleg_full,0)*VLOOKUP(B12,country_opex,3,FALSE))+V12+W12+X12+Y12+Z12)))</f>
         <v/>
       </c>
-      <c r="AX12" s="44" t="inlineStr">
-        <is>
-          <t>PREMIUM tier (nearest comparable = Algeciras&lt;-&gt;Ceuta fast ferry): avg foot-passenger fare ~EUR 33 x 1.08 ~= $36 (one-way ~EUR 25-35), 60 min fast ferry.</t>
-        </is>
-      </c>
+      <c r="AX12" s="44" t="n"/>
       <c r="AY12" s="44" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="29" t="inlineStr">
         <is>
-          <t>Yassir Morocco</t>
+          <t>Yassir</t>
         </is>
       </c>
       <c r="B13" s="29" t="inlineStr">
@@ -3921,11 +3921,11 @@
       </c>
       <c r="C13" s="30" t="inlineStr">
         <is>
-          <t>Casablanca → Rabat</t>
+          <t>Casablanca → Mohammedia</t>
         </is>
       </c>
       <c r="D13" s="31" t="n">
-        <v>46</v>
+        <v>13</v>
       </c>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="32" t="n"/>
@@ -4029,9 +4029,7 @@
         <f>((D13*O13/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D13*O13*VLOOKUP(B13,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG13" s="31" t="n">
-        <v>165000</v>
-      </c>
+      <c r="AG13" s="31" t="n"/>
       <c r="AH13" s="32" t="n"/>
       <c r="AI13" s="32" t="n"/>
       <c r="AJ13" s="39" t="n">
@@ -4084,21 +4082,21 @@
     <row r="14">
       <c r="A14" s="29" t="inlineStr">
         <is>
-          <t>Yassir Tunisia</t>
+          <t>Yassir</t>
         </is>
       </c>
       <c r="B14" s="29" t="inlineStr">
         <is>
-          <t>Tunisia</t>
+          <t>Morocco</t>
         </is>
       </c>
       <c r="C14" s="30" t="inlineStr">
         <is>
-          <t>Jorf (mainland) → Ajim (Djerba Island)</t>
+          <t>Al Hoceima → Cala Iris</t>
         </is>
       </c>
       <c r="D14" s="31" t="n">
-        <v>1.1</v>
+        <v>16</v>
       </c>
       <c r="E14" s="26" t="n"/>
       <c r="F14" s="32" t="n"/>
@@ -4115,7 +4113,7 @@
         <v/>
       </c>
       <c r="K14" s="34">
-        <f>MIN(15,FLOOR(60*service_hr/J14,1))</f>
+        <f>MIN(24,FLOOR(60*service_hr/J14,1))</f>
         <v/>
       </c>
       <c r="L14" s="34">
@@ -4202,9 +4200,7 @@
         <f>((D14*O14/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D14*O14*VLOOKUP(B14,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG14" s="31" t="n">
-        <v>2463750</v>
-      </c>
+      <c r="AG14" s="31" t="n"/>
       <c r="AH14" s="32" t="n"/>
       <c r="AI14" s="32" t="n"/>
       <c r="AJ14" s="39" t="n">
@@ -4257,24 +4253,24 @@
     <row r="15">
       <c r="A15" s="29" t="inlineStr">
         <is>
-          <t>Yassir Tunisia</t>
+          <t>Yassir</t>
         </is>
       </c>
       <c r="B15" s="29" t="inlineStr">
         <is>
-          <t>Tunisia</t>
+          <t>Morocco</t>
         </is>
       </c>
       <c r="C15" s="30" t="inlineStr">
         <is>
-          <t>La Goulette → Sidi Bou Said</t>
+          <t>Tanger Med → Ceuta (Spanish enclave)</t>
         </is>
       </c>
       <c r="D15" s="31" t="n">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="E15" s="26" t="n">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="F15" s="32" t="inlineStr">
         <is>
@@ -4385,9 +4381,7 @@
         <f>((D15*O15/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D15*O15*VLOOKUP(B15,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG15" s="31" t="n">
-        <v>222000</v>
-      </c>
+      <c r="AG15" s="31" t="n"/>
       <c r="AH15" s="32" t="n"/>
       <c r="AI15" s="32" t="n"/>
       <c r="AJ15" s="39" t="n">
@@ -4416,7 +4410,7 @@
       <c r="AP15" s="40" t="n"/>
       <c r="AQ15" s="32" t="inlineStr">
         <is>
-          <t>Grounded</t>
+          <t>Estimated</t>
         </is>
       </c>
       <c r="AR15" s="41" t="n"/>
@@ -4436,7 +4430,7 @@
       </c>
       <c r="AX15" s="44" t="inlineStr">
         <is>
-          <t>PREMIUM charter-divided tier: Gulf of Tunis / Sidi Bou Said per-seat excursion cruise ~EUR 25 (pirate-boat dinner cruise 'from EUR 30'; 3h marina cruise EUR 15-20) x 1.08 ~= $27. Nearest premium per-seat water product on this corridor; no scheduled fast catamaran exists.</t>
+          <t>PREMIUM tier (nearest comparable = Algeciras&lt;-&gt;Ceuta fast ferry): avg foot-passenger fare ~EUR 33 x 1.08 ~= $36 (one-way ~EUR 25-35), 60 min fast ferry.</t>
         </is>
       </c>
       <c r="AY15" s="44" t="n"/>
@@ -4444,21 +4438,21 @@
     <row r="16">
       <c r="A16" s="29" t="inlineStr">
         <is>
-          <t>Yassir Tunisia</t>
+          <t>Yassir</t>
         </is>
       </c>
       <c r="B16" s="29" t="inlineStr">
         <is>
-          <t>Tunisia</t>
+          <t>Morocco</t>
         </is>
       </c>
       <c r="C16" s="30" t="inlineStr">
         <is>
-          <t>Tunis (Tunis Marine) → La Goulette</t>
+          <t>Casablanca → Rabat</t>
         </is>
       </c>
       <c r="D16" s="31" t="n">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="E16" s="26" t="n"/>
       <c r="F16" s="32" t="n"/>
@@ -4563,7 +4557,7 @@
         <v/>
       </c>
       <c r="AG16" s="31" t="n">
-        <v>296000</v>
+        <v>165000</v>
       </c>
       <c r="AH16" s="32" t="n"/>
       <c r="AI16" s="32" t="n"/>
@@ -4593,7 +4587,7 @@
       <c r="AP16" s="40" t="n"/>
       <c r="AQ16" s="32" t="inlineStr">
         <is>
-          <t>Estimated</t>
+          <t>Grounded</t>
         </is>
       </c>
       <c r="AR16" s="41" t="n"/>
@@ -4617,25 +4611,35 @@
     <row r="17">
       <c r="A17" s="29" t="inlineStr">
         <is>
-          <t>Yassir Tunisia</t>
+          <t>Yassir</t>
         </is>
       </c>
       <c r="B17" s="29" t="inlineStr">
         <is>
-          <t>Tunisia</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="C17" s="30" t="inlineStr">
         <is>
-          <t>Tunis (La Goulette) → La Marsa / Gammarth</t>
+          <t>Dakar (Plage de Ngor) → Ile de Ngor</t>
         </is>
       </c>
       <c r="D17" s="31" t="n">
-        <v>7</v>
-      </c>
-      <c r="E17" s="26" t="n"/>
-      <c r="F17" s="32" t="n"/>
-      <c r="G17" s="32" t="n"/>
+        <v>0.3</v>
+      </c>
+      <c r="E17" s="26" t="n">
+        <v>18</v>
+      </c>
+      <c r="F17" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G17" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
       <c r="H17" s="19" t="n">
         <v>1</v>
       </c>
@@ -4648,7 +4652,7 @@
         <v/>
       </c>
       <c r="K17" s="34">
-        <f>MIN(24,FLOOR(60*service_hr/J17,1))</f>
+        <f>MIN(15,FLOOR(60*service_hr/J17,1))</f>
         <v/>
       </c>
       <c r="L17" s="34">
@@ -4735,9 +4739,7 @@
         <f>((D17*O17/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D17*O17*VLOOKUP(B17,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG17" s="31" t="n">
-        <v>222000</v>
-      </c>
+      <c r="AG17" s="31" t="n"/>
       <c r="AH17" s="32" t="n"/>
       <c r="AI17" s="32" t="n"/>
       <c r="AJ17" s="39" t="n">
@@ -4784,30 +4786,34 @@
         <f>IF(((S17*pax_cap*load_full*ROUND(K17*L17*revleg_full,0))-(((battery/range_nm)*D17*ROUND(K17*L17*revleg_full,0)*VLOOKUP(B17,country_opex,3,FALSE))+V17+W17+X17+Y17+Z17))&lt;=0,"",VLOOKUP(B17,country_opex,7,FALSE)/((S17*pax_cap*load_full*ROUND(K17*L17*revleg_full,0))-(((battery/range_nm)*D17*ROUND(K17*L17*revleg_full,0)*VLOOKUP(B17,country_opex,3,FALSE))+V17+W17+X17+Y17+Z17)))</f>
         <v/>
       </c>
-      <c r="AX17" s="44" t="n"/>
+      <c r="AX17" s="44" t="inlineStr">
+        <is>
+          <t>[LB-255 PREMIUM RE-FARE: subsidized comparable $0.87 lifted to premium on-demand floor $18.0] Pirogue shuttle 1,000 FCFA ALLER-RETOUR =&gt; ~500 one-way =&gt; $0.87. NOTE: this corridor has essentially no premium tier today (single low fare); $0.87 doubles as both anchor and floor.</t>
+        </is>
+      </c>
       <c r="AY17" s="44" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="29" t="inlineStr">
         <is>
-          <t>Yassir Tunisia</t>
+          <t>Yassir</t>
         </is>
       </c>
       <c r="B18" s="29" t="inlineStr">
         <is>
-          <t>Tunisia</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="C18" s="30" t="inlineStr">
         <is>
-          <t>Yasmine Hammamet → Nabeul</t>
+          <t>Dakar (Soumbedioune / Mole) → Parc National des Iles de la Madeleine (Ile aux Serpents/Sarpan)</t>
         </is>
       </c>
       <c r="D18" s="31" t="n">
-        <v>7</v>
+        <v>2.2</v>
       </c>
       <c r="E18" s="26" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F18" s="32" t="inlineStr">
         <is>
@@ -4967,7 +4973,7 @@
       </c>
       <c r="AX18" s="44" t="inlineStr">
         <is>
-          <t>PREMIUM charter-divided tier: Hammamet/Nabeul bay per-seat excursion boat ~EUR 15-25 (3h marina cruise w/ swim stop) -&gt; ~EUR 20 x 1.08 ~= $22. Nearest premium per-seat water product on the bay.</t>
+          <t>[LB-255 PREMIUM RE-FARE: subsidized comparable $3.48 lifted to premium on-demand floor $18.0] Divided-pirogue per-seat: 4,000 FCFA/pers ALLER-RETOUR for the crossing (excl. 1,000 FCFA park entry + 5,000 FCFA/group guide) =&gt; ~2,000 one-way =&gt; $3.48.</t>
         </is>
       </c>
       <c r="AY18" s="44" t="n"/>
@@ -4975,25 +4981,35 @@
     <row r="19">
       <c r="A19" s="29" t="inlineStr">
         <is>
-          <t>Yassir Tunisia</t>
+          <t>Yassir</t>
         </is>
       </c>
       <c r="B19" s="29" t="inlineStr">
         <is>
-          <t>Tunisia</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="C19" s="30" t="inlineStr">
         <is>
-          <t>Sfax → Sidi Youssef (Kerkennah Islands)</t>
+          <t>Dakar Port → Île de Gorée</t>
         </is>
       </c>
       <c r="D19" s="31" t="n">
-        <v>11</v>
-      </c>
-      <c r="E19" s="26" t="n"/>
-      <c r="F19" s="32" t="n"/>
-      <c r="G19" s="32" t="n"/>
+        <v>2.5</v>
+      </c>
+      <c r="E19" s="26" t="n">
+        <v>18</v>
+      </c>
+      <c r="F19" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G19" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
       <c r="H19" s="19" t="n">
         <v>1</v>
       </c>
@@ -5094,12 +5110,16 @@
         <v/>
       </c>
       <c r="AG19" s="31" t="n">
-        <v>1750000</v>
+        <v>80000</v>
       </c>
       <c r="AH19" s="32" t="n"/>
-      <c r="AI19" s="32" t="n"/>
+      <c r="AI19" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
       <c r="AJ19" s="39" t="n">
-        <v>0.1</v>
+        <v>0.25</v>
       </c>
       <c r="AK19" s="34">
         <f>IF(AG19="","",AG19*AJ19)</f>
@@ -5124,7 +5144,7 @@
       <c r="AP19" s="40" t="n"/>
       <c r="AQ19" s="32" t="inlineStr">
         <is>
-          <t>Estimated</t>
+          <t>Grounded</t>
         </is>
       </c>
       <c r="AR19" s="41" t="n"/>
@@ -5142,41 +5162,35 @@
         <f>IF(((S19*pax_cap*load_full*ROUND(K19*L19*revleg_full,0))-(((battery/range_nm)*D19*ROUND(K19*L19*revleg_full,0)*VLOOKUP(B19,country_opex,3,FALSE))+V19+W19+X19+Y19+Z19))&lt;=0,"",VLOOKUP(B19,country_opex,7,FALSE)/((S19*pax_cap*load_full*ROUND(K19*L19*revleg_full,0))-(((battery/range_nm)*D19*ROUND(K19*L19*revleg_full,0)*VLOOKUP(B19,country_opex,3,FALSE))+V19+W19+X19+Y19+Z19)))</f>
         <v/>
       </c>
-      <c r="AX19" s="44" t="n"/>
+      <c r="AX19" s="44" t="inlineStr">
+        <is>
+          <t>[LB-255 PREMIUM RE-FARE: subsidized comparable $5.22 lifted to premium on-demand floor $18.0] PREMIUM tier: non-resident (foreign) adult tourist fare 6,000 FCFA ALLER-RETOUR (effective Oct 2025) =&gt; ~3,000 FCFA one-way =&gt; $5.22. (Pre-Oct-2025 non-resident fare was 5,200 FCFA RT.)</t>
+        </is>
+      </c>
       <c r="AY19" s="44" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="29" t="inlineStr">
         <is>
-          <t>Yassir Tunisia</t>
+          <t>Yassir</t>
         </is>
       </c>
       <c r="B20" s="29" t="inlineStr">
         <is>
-          <t>Tunisia</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="C20" s="30" t="inlineStr">
         <is>
-          <t>Sousse (Port El Kantaoui) → Monastir (Marina)</t>
+          <t>Dakar (Yoff / Almadies) → Dakar (Soumbedioune / Plateau)</t>
         </is>
       </c>
       <c r="D20" s="31" t="n">
-        <v>12</v>
-      </c>
-      <c r="E20" s="26" t="n">
-        <v>32</v>
-      </c>
-      <c r="F20" s="32" t="inlineStr">
-        <is>
-          <t>T2</t>
-        </is>
-      </c>
-      <c r="G20" s="32" t="inlineStr">
-        <is>
-          <t>med</t>
-        </is>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="E20" s="26" t="n"/>
+      <c r="F20" s="32" t="n"/>
+      <c r="G20" s="32" t="n"/>
       <c r="H20" s="19" t="n">
         <v>1</v>
       </c>
@@ -5189,7 +5203,7 @@
         <v/>
       </c>
       <c r="K20" s="34">
-        <f>MIN(24,FLOOR(60*service_hr/J20,1))</f>
+        <f>MIN(15,FLOOR(60*service_hr/J20,1))</f>
         <v/>
       </c>
       <c r="L20" s="34">
@@ -5276,9 +5290,7 @@
         <f>((D20*O20/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D20*O20*VLOOKUP(B20,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG20" s="31" t="n">
-        <v>344000</v>
-      </c>
+      <c r="AG20" s="31" t="n"/>
       <c r="AH20" s="32" t="n"/>
       <c r="AI20" s="32" t="n"/>
       <c r="AJ20" s="39" t="n">
@@ -5307,7 +5319,7 @@
       <c r="AP20" s="40" t="n"/>
       <c r="AQ20" s="32" t="inlineStr">
         <is>
-          <t>Grounded</t>
+          <t>Estimated</t>
         </is>
       </c>
       <c r="AR20" s="41" t="n"/>
@@ -5325,216 +5337,1412 @@
         <f>IF(((S20*pax_cap*load_full*ROUND(K20*L20*revleg_full,0))-(((battery/range_nm)*D20*ROUND(K20*L20*revleg_full,0)*VLOOKUP(B20,country_opex,3,FALSE))+V20+W20+X20+Y20+Z20))&lt;=0,"",VLOOKUP(B20,country_opex,7,FALSE)/((S20*pax_cap*load_full*ROUND(K20*L20*revleg_full,0))-(((battery/range_nm)*D20*ROUND(K20*L20*revleg_full,0)*VLOOKUP(B20,country_opex,3,FALSE))+V20+W20+X20+Y20+Z20)))</f>
         <v/>
       </c>
-      <c r="AX20" s="44" t="inlineStr">
+      <c r="AX20" s="44" t="n"/>
+      <c r="AY20" s="44" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="29" t="inlineStr">
+        <is>
+          <t>Yassir</t>
+        </is>
+      </c>
+      <c r="B21" s="29" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="C21" s="30" t="inlineStr">
+        <is>
+          <t>Dakar / Mbour-Petite Cote → Foundiougne (Sine-Saloum delta)</t>
+        </is>
+      </c>
+      <c r="D21" s="31" t="n">
+        <v>60</v>
+      </c>
+      <c r="E21" s="26" t="n"/>
+      <c r="F21" s="32" t="n"/>
+      <c r="G21" s="32" t="n"/>
+      <c r="H21" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" s="33">
+        <f>60*D21/cruise_kt</f>
+        <v/>
+      </c>
+      <c r="J21" s="33">
+        <f>I21+turn_min+dwell_min</f>
+        <v/>
+      </c>
+      <c r="K21" s="34">
+        <f>MIN(15,FLOOR(60*service_hr/J21,1))</f>
+        <v/>
+      </c>
+      <c r="L21" s="34">
+        <f>ROUND(365*mech_uptime*H21,0)</f>
+        <v/>
+      </c>
+      <c r="M21" s="35">
+        <f>mech_uptime</f>
+        <v/>
+      </c>
+      <c r="N21" s="35">
+        <f>revleg_sel</f>
+        <v/>
+      </c>
+      <c r="O21" s="34">
+        <f>ROUND(K21*L21*revleg_sel,0)</f>
+        <v/>
+      </c>
+      <c r="P21" s="36">
+        <f>load_sel</f>
+        <v/>
+      </c>
+      <c r="Q21" s="36">
+        <f>pax_cap*P21</f>
+        <v/>
+      </c>
+      <c r="R21" s="34">
+        <f>Q21*O21</f>
+        <v/>
+      </c>
+      <c r="S21" s="37">
+        <f>E21*discount</f>
+        <v/>
+      </c>
+      <c r="T21" s="38">
+        <f>S21*R21</f>
+        <v/>
+      </c>
+      <c r="U21" s="38">
+        <f>(battery/range_nm)*D21*O21*VLOOKUP(B21,country_opex,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="V21" s="38">
+        <f>VLOOKUP(B21,country_opex,2,FALSE)*crew_factor</f>
+        <v/>
+      </c>
+      <c r="W21" s="38">
+        <f>VLOOKUP(B21,country_opex,5,FALSE)</f>
+        <v/>
+      </c>
+      <c r="X21" s="38">
+        <f>maint</f>
+        <v/>
+      </c>
+      <c r="Y21" s="38">
+        <f>VLOOKUP(B21,country_opex,7,FALSE)*ins_pct</f>
+        <v/>
+      </c>
+      <c r="Z21" s="38">
+        <f>charge_berth</f>
+        <v/>
+      </c>
+      <c r="AA21" s="38">
+        <f>U21+V21+W21+X21+Y21+Z21</f>
+        <v/>
+      </c>
+      <c r="AB21" s="38">
+        <f>VLOOKUP(B21,country_opex,7,FALSE)/dep_years</f>
+        <v/>
+      </c>
+      <c r="AC21" s="38">
+        <f>T21-AA21</f>
+        <v/>
+      </c>
+      <c r="AD21" s="35">
+        <f>IF(T21=0,"",AC21/T21)</f>
+        <v/>
+      </c>
+      <c r="AE21" s="36">
+        <f>IF(AC21&lt;=0,"",VLOOKUP(B21,country_opex,7,FALSE)/AC21)</f>
+        <v/>
+      </c>
+      <c r="AF21" s="33">
+        <f>((D21*O21/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D21*O21*VLOOKUP(B21,country_opex,4,FALSE))/1000</f>
+        <v/>
+      </c>
+      <c r="AG21" s="31" t="n"/>
+      <c r="AH21" s="32" t="n"/>
+      <c r="AI21" s="32" t="n"/>
+      <c r="AJ21" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AK21" s="34">
+        <f>IF(AG21="","",AG21*AJ21)</f>
+        <v/>
+      </c>
+      <c r="AL21" s="34">
+        <f>IF(OR(AG21="",R21=0),"",MIN(IF(AT21="",9.9E+99,AT21),FLOOR(AK21/R21,1)))</f>
+        <v/>
+      </c>
+      <c r="AM21" s="38">
+        <f>IF(AL21="","",AL21*T21)</f>
+        <v/>
+      </c>
+      <c r="AN21" s="36">
+        <f>IF(OR(AG21="",R21=0),"",MIN(IF(AT21="",9.9E+99,AT21),AK21/R21))</f>
+        <v/>
+      </c>
+      <c r="AO21" s="38">
+        <f>IF(AN21="","",AN21*T21)</f>
+        <v/>
+      </c>
+      <c r="AP21" s="40" t="n"/>
+      <c r="AQ21" s="32" t="inlineStr">
+        <is>
+          <t>Estimated</t>
+        </is>
+      </c>
+      <c r="AR21" s="41" t="n"/>
+      <c r="AS21" s="41" t="n"/>
+      <c r="AT21" s="42" t="n"/>
+      <c r="AU21" s="43">
+        <f>IF(((S21*pax_cap*load_thin*ROUND(K21*L21*revleg_thin,0))-(((battery/range_nm)*D21*ROUND(K21*L21*revleg_thin,0)*VLOOKUP(B21,country_opex,3,FALSE))+V21+W21+X21+Y21+Z21))&lt;=0,"",VLOOKUP(B21,country_opex,7,FALSE)/((S21*pax_cap*load_thin*ROUND(K21*L21*revleg_thin,0))-(((battery/range_nm)*D21*ROUND(K21*L21*revleg_thin,0)*VLOOKUP(B21,country_opex,3,FALSE))+V21+W21+X21+Y21+Z21)))</f>
+        <v/>
+      </c>
+      <c r="AV21" s="43">
+        <f>IF(((S21*pax_cap*load_mid*ROUND(K21*L21*revleg_mid,0))-(((battery/range_nm)*D21*ROUND(K21*L21*revleg_mid,0)*VLOOKUP(B21,country_opex,3,FALSE))+V21+W21+X21+Y21+Z21))&lt;=0,"",VLOOKUP(B21,country_opex,7,FALSE)/((S21*pax_cap*load_mid*ROUND(K21*L21*revleg_mid,0))-(((battery/range_nm)*D21*ROUND(K21*L21*revleg_mid,0)*VLOOKUP(B21,country_opex,3,FALSE))+V21+W21+X21+Y21+Z21)))</f>
+        <v/>
+      </c>
+      <c r="AW21" s="43">
+        <f>IF(((S21*pax_cap*load_full*ROUND(K21*L21*revleg_full,0))-(((battery/range_nm)*D21*ROUND(K21*L21*revleg_full,0)*VLOOKUP(B21,country_opex,3,FALSE))+V21+W21+X21+Y21+Z21))&lt;=0,"",VLOOKUP(B21,country_opex,7,FALSE)/((S21*pax_cap*load_full*ROUND(K21*L21*revleg_full,0))-(((battery/range_nm)*D21*ROUND(K21*L21*revleg_full,0)*VLOOKUP(B21,country_opex,3,FALSE))+V21+W21+X21+Y21+Z21)))</f>
+        <v/>
+      </c>
+      <c r="AX21" s="44" t="n"/>
+      <c r="AY21" s="44" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="29" t="inlineStr">
+        <is>
+          <t>Yassir</t>
+        </is>
+      </c>
+      <c r="B22" s="29" t="inlineStr">
+        <is>
+          <t>Tunisia</t>
+        </is>
+      </c>
+      <c r="C22" s="30" t="inlineStr">
+        <is>
+          <t>Jorf (mainland) → Ajim (Djerba Island)</t>
+        </is>
+      </c>
+      <c r="D22" s="31" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E22" s="26" t="n"/>
+      <c r="F22" s="32" t="n"/>
+      <c r="G22" s="32" t="n"/>
+      <c r="H22" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" s="33">
+        <f>60*D22/cruise_kt</f>
+        <v/>
+      </c>
+      <c r="J22" s="33">
+        <f>I22+turn_min+dwell_min</f>
+        <v/>
+      </c>
+      <c r="K22" s="34">
+        <f>MIN(15,FLOOR(60*service_hr/J22,1))</f>
+        <v/>
+      </c>
+      <c r="L22" s="34">
+        <f>ROUND(365*mech_uptime*H22,0)</f>
+        <v/>
+      </c>
+      <c r="M22" s="35">
+        <f>mech_uptime</f>
+        <v/>
+      </c>
+      <c r="N22" s="35">
+        <f>revleg_sel</f>
+        <v/>
+      </c>
+      <c r="O22" s="34">
+        <f>ROUND(K22*L22*revleg_sel,0)</f>
+        <v/>
+      </c>
+      <c r="P22" s="36">
+        <f>load_sel</f>
+        <v/>
+      </c>
+      <c r="Q22" s="36">
+        <f>pax_cap*P22</f>
+        <v/>
+      </c>
+      <c r="R22" s="34">
+        <f>Q22*O22</f>
+        <v/>
+      </c>
+      <c r="S22" s="37">
+        <f>E22*discount</f>
+        <v/>
+      </c>
+      <c r="T22" s="38">
+        <f>S22*R22</f>
+        <v/>
+      </c>
+      <c r="U22" s="38">
+        <f>(battery/range_nm)*D22*O22*VLOOKUP(B22,country_opex,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="V22" s="38">
+        <f>VLOOKUP(B22,country_opex,2,FALSE)*crew_factor</f>
+        <v/>
+      </c>
+      <c r="W22" s="38">
+        <f>VLOOKUP(B22,country_opex,5,FALSE)</f>
+        <v/>
+      </c>
+      <c r="X22" s="38">
+        <f>maint</f>
+        <v/>
+      </c>
+      <c r="Y22" s="38">
+        <f>VLOOKUP(B22,country_opex,7,FALSE)*ins_pct</f>
+        <v/>
+      </c>
+      <c r="Z22" s="38">
+        <f>charge_berth</f>
+        <v/>
+      </c>
+      <c r="AA22" s="38">
+        <f>U22+V22+W22+X22+Y22+Z22</f>
+        <v/>
+      </c>
+      <c r="AB22" s="38">
+        <f>VLOOKUP(B22,country_opex,7,FALSE)/dep_years</f>
+        <v/>
+      </c>
+      <c r="AC22" s="38">
+        <f>T22-AA22</f>
+        <v/>
+      </c>
+      <c r="AD22" s="35">
+        <f>IF(T22=0,"",AC22/T22)</f>
+        <v/>
+      </c>
+      <c r="AE22" s="36">
+        <f>IF(AC22&lt;=0,"",VLOOKUP(B22,country_opex,7,FALSE)/AC22)</f>
+        <v/>
+      </c>
+      <c r="AF22" s="33">
+        <f>((D22*O22/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D22*O22*VLOOKUP(B22,country_opex,4,FALSE))/1000</f>
+        <v/>
+      </c>
+      <c r="AG22" s="31" t="n">
+        <v>2463750</v>
+      </c>
+      <c r="AH22" s="32" t="n"/>
+      <c r="AI22" s="32" t="n"/>
+      <c r="AJ22" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AK22" s="34">
+        <f>IF(AG22="","",AG22*AJ22)</f>
+        <v/>
+      </c>
+      <c r="AL22" s="34">
+        <f>IF(OR(AG22="",R22=0),"",MIN(IF(AT22="",9.9E+99,AT22),FLOOR(AK22/R22,1)))</f>
+        <v/>
+      </c>
+      <c r="AM22" s="38">
+        <f>IF(AL22="","",AL22*T22)</f>
+        <v/>
+      </c>
+      <c r="AN22" s="36">
+        <f>IF(OR(AG22="",R22=0),"",MIN(IF(AT22="",9.9E+99,AT22),AK22/R22))</f>
+        <v/>
+      </c>
+      <c r="AO22" s="38">
+        <f>IF(AN22="","",AN22*T22)</f>
+        <v/>
+      </c>
+      <c r="AP22" s="40" t="n"/>
+      <c r="AQ22" s="32" t="inlineStr">
+        <is>
+          <t>Grounded</t>
+        </is>
+      </c>
+      <c r="AR22" s="41" t="n"/>
+      <c r="AS22" s="41" t="n"/>
+      <c r="AT22" s="42" t="n"/>
+      <c r="AU22" s="43">
+        <f>IF(((S22*pax_cap*load_thin*ROUND(K22*L22*revleg_thin,0))-(((battery/range_nm)*D22*ROUND(K22*L22*revleg_thin,0)*VLOOKUP(B22,country_opex,3,FALSE))+V22+W22+X22+Y22+Z22))&lt;=0,"",VLOOKUP(B22,country_opex,7,FALSE)/((S22*pax_cap*load_thin*ROUND(K22*L22*revleg_thin,0))-(((battery/range_nm)*D22*ROUND(K22*L22*revleg_thin,0)*VLOOKUP(B22,country_opex,3,FALSE))+V22+W22+X22+Y22+Z22)))</f>
+        <v/>
+      </c>
+      <c r="AV22" s="43">
+        <f>IF(((S22*pax_cap*load_mid*ROUND(K22*L22*revleg_mid,0))-(((battery/range_nm)*D22*ROUND(K22*L22*revleg_mid,0)*VLOOKUP(B22,country_opex,3,FALSE))+V22+W22+X22+Y22+Z22))&lt;=0,"",VLOOKUP(B22,country_opex,7,FALSE)/((S22*pax_cap*load_mid*ROUND(K22*L22*revleg_mid,0))-(((battery/range_nm)*D22*ROUND(K22*L22*revleg_mid,0)*VLOOKUP(B22,country_opex,3,FALSE))+V22+W22+X22+Y22+Z22)))</f>
+        <v/>
+      </c>
+      <c r="AW22" s="43">
+        <f>IF(((S22*pax_cap*load_full*ROUND(K22*L22*revleg_full,0))-(((battery/range_nm)*D22*ROUND(K22*L22*revleg_full,0)*VLOOKUP(B22,country_opex,3,FALSE))+V22+W22+X22+Y22+Z22))&lt;=0,"",VLOOKUP(B22,country_opex,7,FALSE)/((S22*pax_cap*load_full*ROUND(K22*L22*revleg_full,0))-(((battery/range_nm)*D22*ROUND(K22*L22*revleg_full,0)*VLOOKUP(B22,country_opex,3,FALSE))+V22+W22+X22+Y22+Z22)))</f>
+        <v/>
+      </c>
+      <c r="AX22" s="44" t="n"/>
+      <c r="AY22" s="44" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="29" t="inlineStr">
+        <is>
+          <t>Yassir</t>
+        </is>
+      </c>
+      <c r="B23" s="29" t="inlineStr">
+        <is>
+          <t>Tunisia</t>
+        </is>
+      </c>
+      <c r="C23" s="30" t="inlineStr">
+        <is>
+          <t>La Goulette → Sidi Bou Said</t>
+        </is>
+      </c>
+      <c r="D23" s="31" t="n">
+        <v>4</v>
+      </c>
+      <c r="E23" s="26" t="n">
+        <v>27</v>
+      </c>
+      <c r="F23" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G23" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="H23" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" s="33">
+        <f>60*D23/cruise_kt</f>
+        <v/>
+      </c>
+      <c r="J23" s="33">
+        <f>I23+turn_min+dwell_min</f>
+        <v/>
+      </c>
+      <c r="K23" s="34">
+        <f>MIN(15,FLOOR(60*service_hr/J23,1))</f>
+        <v/>
+      </c>
+      <c r="L23" s="34">
+        <f>ROUND(365*mech_uptime*H23,0)</f>
+        <v/>
+      </c>
+      <c r="M23" s="35">
+        <f>mech_uptime</f>
+        <v/>
+      </c>
+      <c r="N23" s="35">
+        <f>revleg_sel</f>
+        <v/>
+      </c>
+      <c r="O23" s="34">
+        <f>ROUND(K23*L23*revleg_sel,0)</f>
+        <v/>
+      </c>
+      <c r="P23" s="36">
+        <f>load_sel</f>
+        <v/>
+      </c>
+      <c r="Q23" s="36">
+        <f>pax_cap*P23</f>
+        <v/>
+      </c>
+      <c r="R23" s="34">
+        <f>Q23*O23</f>
+        <v/>
+      </c>
+      <c r="S23" s="37">
+        <f>E23*discount</f>
+        <v/>
+      </c>
+      <c r="T23" s="38">
+        <f>S23*R23</f>
+        <v/>
+      </c>
+      <c r="U23" s="38">
+        <f>(battery/range_nm)*D23*O23*VLOOKUP(B23,country_opex,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="V23" s="38">
+        <f>VLOOKUP(B23,country_opex,2,FALSE)*crew_factor</f>
+        <v/>
+      </c>
+      <c r="W23" s="38">
+        <f>VLOOKUP(B23,country_opex,5,FALSE)</f>
+        <v/>
+      </c>
+      <c r="X23" s="38">
+        <f>maint</f>
+        <v/>
+      </c>
+      <c r="Y23" s="38">
+        <f>VLOOKUP(B23,country_opex,7,FALSE)*ins_pct</f>
+        <v/>
+      </c>
+      <c r="Z23" s="38">
+        <f>charge_berth</f>
+        <v/>
+      </c>
+      <c r="AA23" s="38">
+        <f>U23+V23+W23+X23+Y23+Z23</f>
+        <v/>
+      </c>
+      <c r="AB23" s="38">
+        <f>VLOOKUP(B23,country_opex,7,FALSE)/dep_years</f>
+        <v/>
+      </c>
+      <c r="AC23" s="38">
+        <f>T23-AA23</f>
+        <v/>
+      </c>
+      <c r="AD23" s="35">
+        <f>IF(T23=0,"",AC23/T23)</f>
+        <v/>
+      </c>
+      <c r="AE23" s="36">
+        <f>IF(AC23&lt;=0,"",VLOOKUP(B23,country_opex,7,FALSE)/AC23)</f>
+        <v/>
+      </c>
+      <c r="AF23" s="33">
+        <f>((D23*O23/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D23*O23*VLOOKUP(B23,country_opex,4,FALSE))/1000</f>
+        <v/>
+      </c>
+      <c r="AG23" s="31" t="n">
+        <v>222000</v>
+      </c>
+      <c r="AH23" s="32" t="n"/>
+      <c r="AI23" s="32" t="n"/>
+      <c r="AJ23" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AK23" s="34">
+        <f>IF(AG23="","",AG23*AJ23)</f>
+        <v/>
+      </c>
+      <c r="AL23" s="34">
+        <f>IF(OR(AG23="",R23=0),"",MIN(IF(AT23="",9.9E+99,AT23),FLOOR(AK23/R23,1)))</f>
+        <v/>
+      </c>
+      <c r="AM23" s="38">
+        <f>IF(AL23="","",AL23*T23)</f>
+        <v/>
+      </c>
+      <c r="AN23" s="36">
+        <f>IF(OR(AG23="",R23=0),"",MIN(IF(AT23="",9.9E+99,AT23),AK23/R23))</f>
+        <v/>
+      </c>
+      <c r="AO23" s="38">
+        <f>IF(AN23="","",AN23*T23)</f>
+        <v/>
+      </c>
+      <c r="AP23" s="40" t="n"/>
+      <c r="AQ23" s="32" t="inlineStr">
+        <is>
+          <t>Grounded</t>
+        </is>
+      </c>
+      <c r="AR23" s="41" t="n"/>
+      <c r="AS23" s="41" t="n"/>
+      <c r="AT23" s="42" t="n"/>
+      <c r="AU23" s="43">
+        <f>IF(((S23*pax_cap*load_thin*ROUND(K23*L23*revleg_thin,0))-(((battery/range_nm)*D23*ROUND(K23*L23*revleg_thin,0)*VLOOKUP(B23,country_opex,3,FALSE))+V23+W23+X23+Y23+Z23))&lt;=0,"",VLOOKUP(B23,country_opex,7,FALSE)/((S23*pax_cap*load_thin*ROUND(K23*L23*revleg_thin,0))-(((battery/range_nm)*D23*ROUND(K23*L23*revleg_thin,0)*VLOOKUP(B23,country_opex,3,FALSE))+V23+W23+X23+Y23+Z23)))</f>
+        <v/>
+      </c>
+      <c r="AV23" s="43">
+        <f>IF(((S23*pax_cap*load_mid*ROUND(K23*L23*revleg_mid,0))-(((battery/range_nm)*D23*ROUND(K23*L23*revleg_mid,0)*VLOOKUP(B23,country_opex,3,FALSE))+V23+W23+X23+Y23+Z23))&lt;=0,"",VLOOKUP(B23,country_opex,7,FALSE)/((S23*pax_cap*load_mid*ROUND(K23*L23*revleg_mid,0))-(((battery/range_nm)*D23*ROUND(K23*L23*revleg_mid,0)*VLOOKUP(B23,country_opex,3,FALSE))+V23+W23+X23+Y23+Z23)))</f>
+        <v/>
+      </c>
+      <c r="AW23" s="43">
+        <f>IF(((S23*pax_cap*load_full*ROUND(K23*L23*revleg_full,0))-(((battery/range_nm)*D23*ROUND(K23*L23*revleg_full,0)*VLOOKUP(B23,country_opex,3,FALSE))+V23+W23+X23+Y23+Z23))&lt;=0,"",VLOOKUP(B23,country_opex,7,FALSE)/((S23*pax_cap*load_full*ROUND(K23*L23*revleg_full,0))-(((battery/range_nm)*D23*ROUND(K23*L23*revleg_full,0)*VLOOKUP(B23,country_opex,3,FALSE))+V23+W23+X23+Y23+Z23)))</f>
+        <v/>
+      </c>
+      <c r="AX23" s="44" t="inlineStr">
+        <is>
+          <t>PREMIUM charter-divided tier: Gulf of Tunis / Sidi Bou Said per-seat excursion cruise ~EUR 25 (pirate-boat dinner cruise 'from EUR 30'; 3h marina cruise EUR 15-20) x 1.08 ~= $27. Nearest premium per-seat water product on this corridor; no scheduled fast catamaran exists.</t>
+        </is>
+      </c>
+      <c r="AY23" s="44" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="29" t="inlineStr">
+        <is>
+          <t>Yassir</t>
+        </is>
+      </c>
+      <c r="B24" s="29" t="inlineStr">
+        <is>
+          <t>Tunisia</t>
+        </is>
+      </c>
+      <c r="C24" s="30" t="inlineStr">
+        <is>
+          <t>Tunis (Tunis Marine) → La Goulette</t>
+        </is>
+      </c>
+      <c r="D24" s="31" t="n">
+        <v>5</v>
+      </c>
+      <c r="E24" s="26" t="n"/>
+      <c r="F24" s="32" t="n"/>
+      <c r="G24" s="32" t="n"/>
+      <c r="H24" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" s="33">
+        <f>60*D24/cruise_kt</f>
+        <v/>
+      </c>
+      <c r="J24" s="33">
+        <f>I24+turn_min+dwell_min</f>
+        <v/>
+      </c>
+      <c r="K24" s="34">
+        <f>MIN(24,FLOOR(60*service_hr/J24,1))</f>
+        <v/>
+      </c>
+      <c r="L24" s="34">
+        <f>ROUND(365*mech_uptime*H24,0)</f>
+        <v/>
+      </c>
+      <c r="M24" s="35">
+        <f>mech_uptime</f>
+        <v/>
+      </c>
+      <c r="N24" s="35">
+        <f>revleg_sel</f>
+        <v/>
+      </c>
+      <c r="O24" s="34">
+        <f>ROUND(K24*L24*revleg_sel,0)</f>
+        <v/>
+      </c>
+      <c r="P24" s="36">
+        <f>load_sel</f>
+        <v/>
+      </c>
+      <c r="Q24" s="36">
+        <f>pax_cap*P24</f>
+        <v/>
+      </c>
+      <c r="R24" s="34">
+        <f>Q24*O24</f>
+        <v/>
+      </c>
+      <c r="S24" s="37">
+        <f>E24*discount</f>
+        <v/>
+      </c>
+      <c r="T24" s="38">
+        <f>S24*R24</f>
+        <v/>
+      </c>
+      <c r="U24" s="38">
+        <f>(battery/range_nm)*D24*O24*VLOOKUP(B24,country_opex,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="V24" s="38">
+        <f>VLOOKUP(B24,country_opex,2,FALSE)*crew_factor</f>
+        <v/>
+      </c>
+      <c r="W24" s="38">
+        <f>VLOOKUP(B24,country_opex,5,FALSE)</f>
+        <v/>
+      </c>
+      <c r="X24" s="38">
+        <f>maint</f>
+        <v/>
+      </c>
+      <c r="Y24" s="38">
+        <f>VLOOKUP(B24,country_opex,7,FALSE)*ins_pct</f>
+        <v/>
+      </c>
+      <c r="Z24" s="38">
+        <f>charge_berth</f>
+        <v/>
+      </c>
+      <c r="AA24" s="38">
+        <f>U24+V24+W24+X24+Y24+Z24</f>
+        <v/>
+      </c>
+      <c r="AB24" s="38">
+        <f>VLOOKUP(B24,country_opex,7,FALSE)/dep_years</f>
+        <v/>
+      </c>
+      <c r="AC24" s="38">
+        <f>T24-AA24</f>
+        <v/>
+      </c>
+      <c r="AD24" s="35">
+        <f>IF(T24=0,"",AC24/T24)</f>
+        <v/>
+      </c>
+      <c r="AE24" s="36">
+        <f>IF(AC24&lt;=0,"",VLOOKUP(B24,country_opex,7,FALSE)/AC24)</f>
+        <v/>
+      </c>
+      <c r="AF24" s="33">
+        <f>((D24*O24/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D24*O24*VLOOKUP(B24,country_opex,4,FALSE))/1000</f>
+        <v/>
+      </c>
+      <c r="AG24" s="31" t="n">
+        <v>296000</v>
+      </c>
+      <c r="AH24" s="32" t="n"/>
+      <c r="AI24" s="32" t="n"/>
+      <c r="AJ24" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AK24" s="34">
+        <f>IF(AG24="","",AG24*AJ24)</f>
+        <v/>
+      </c>
+      <c r="AL24" s="34">
+        <f>IF(OR(AG24="",R24=0),"",MIN(IF(AT24="",9.9E+99,AT24),FLOOR(AK24/R24,1)))</f>
+        <v/>
+      </c>
+      <c r="AM24" s="38">
+        <f>IF(AL24="","",AL24*T24)</f>
+        <v/>
+      </c>
+      <c r="AN24" s="36">
+        <f>IF(OR(AG24="",R24=0),"",MIN(IF(AT24="",9.9E+99,AT24),AK24/R24))</f>
+        <v/>
+      </c>
+      <c r="AO24" s="38">
+        <f>IF(AN24="","",AN24*T24)</f>
+        <v/>
+      </c>
+      <c r="AP24" s="40" t="n"/>
+      <c r="AQ24" s="32" t="inlineStr">
+        <is>
+          <t>Grounded</t>
+        </is>
+      </c>
+      <c r="AR24" s="41" t="n"/>
+      <c r="AS24" s="41" t="n"/>
+      <c r="AT24" s="42" t="n"/>
+      <c r="AU24" s="43">
+        <f>IF(((S24*pax_cap*load_thin*ROUND(K24*L24*revleg_thin,0))-(((battery/range_nm)*D24*ROUND(K24*L24*revleg_thin,0)*VLOOKUP(B24,country_opex,3,FALSE))+V24+W24+X24+Y24+Z24))&lt;=0,"",VLOOKUP(B24,country_opex,7,FALSE)/((S24*pax_cap*load_thin*ROUND(K24*L24*revleg_thin,0))-(((battery/range_nm)*D24*ROUND(K24*L24*revleg_thin,0)*VLOOKUP(B24,country_opex,3,FALSE))+V24+W24+X24+Y24+Z24)))</f>
+        <v/>
+      </c>
+      <c r="AV24" s="43">
+        <f>IF(((S24*pax_cap*load_mid*ROUND(K24*L24*revleg_mid,0))-(((battery/range_nm)*D24*ROUND(K24*L24*revleg_mid,0)*VLOOKUP(B24,country_opex,3,FALSE))+V24+W24+X24+Y24+Z24))&lt;=0,"",VLOOKUP(B24,country_opex,7,FALSE)/((S24*pax_cap*load_mid*ROUND(K24*L24*revleg_mid,0))-(((battery/range_nm)*D24*ROUND(K24*L24*revleg_mid,0)*VLOOKUP(B24,country_opex,3,FALSE))+V24+W24+X24+Y24+Z24)))</f>
+        <v/>
+      </c>
+      <c r="AW24" s="43">
+        <f>IF(((S24*pax_cap*load_full*ROUND(K24*L24*revleg_full,0))-(((battery/range_nm)*D24*ROUND(K24*L24*revleg_full,0)*VLOOKUP(B24,country_opex,3,FALSE))+V24+W24+X24+Y24+Z24))&lt;=0,"",VLOOKUP(B24,country_opex,7,FALSE)/((S24*pax_cap*load_full*ROUND(K24*L24*revleg_full,0))-(((battery/range_nm)*D24*ROUND(K24*L24*revleg_full,0)*VLOOKUP(B24,country_opex,3,FALSE))+V24+W24+X24+Y24+Z24)))</f>
+        <v/>
+      </c>
+      <c r="AX24" s="44" t="n"/>
+      <c r="AY24" s="44" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="29" t="inlineStr">
+        <is>
+          <t>Yassir</t>
+        </is>
+      </c>
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>Tunisia</t>
+        </is>
+      </c>
+      <c r="C25" s="30" t="inlineStr">
+        <is>
+          <t>Tunis (La Goulette) → La Marsa / Gammarth</t>
+        </is>
+      </c>
+      <c r="D25" s="31" t="n">
+        <v>7</v>
+      </c>
+      <c r="E25" s="26" t="n"/>
+      <c r="F25" s="32" t="n"/>
+      <c r="G25" s="32" t="n"/>
+      <c r="H25" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I25" s="33">
+        <f>60*D25/cruise_kt</f>
+        <v/>
+      </c>
+      <c r="J25" s="33">
+        <f>I25+turn_min+dwell_min</f>
+        <v/>
+      </c>
+      <c r="K25" s="34">
+        <f>MIN(24,FLOOR(60*service_hr/J25,1))</f>
+        <v/>
+      </c>
+      <c r="L25" s="34">
+        <f>ROUND(365*mech_uptime*H25,0)</f>
+        <v/>
+      </c>
+      <c r="M25" s="35">
+        <f>mech_uptime</f>
+        <v/>
+      </c>
+      <c r="N25" s="35">
+        <f>revleg_sel</f>
+        <v/>
+      </c>
+      <c r="O25" s="34">
+        <f>ROUND(K25*L25*revleg_sel,0)</f>
+        <v/>
+      </c>
+      <c r="P25" s="36">
+        <f>load_sel</f>
+        <v/>
+      </c>
+      <c r="Q25" s="36">
+        <f>pax_cap*P25</f>
+        <v/>
+      </c>
+      <c r="R25" s="34">
+        <f>Q25*O25</f>
+        <v/>
+      </c>
+      <c r="S25" s="37">
+        <f>E25*discount</f>
+        <v/>
+      </c>
+      <c r="T25" s="38">
+        <f>S25*R25</f>
+        <v/>
+      </c>
+      <c r="U25" s="38">
+        <f>(battery/range_nm)*D25*O25*VLOOKUP(B25,country_opex,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="V25" s="38">
+        <f>VLOOKUP(B25,country_opex,2,FALSE)*crew_factor</f>
+        <v/>
+      </c>
+      <c r="W25" s="38">
+        <f>VLOOKUP(B25,country_opex,5,FALSE)</f>
+        <v/>
+      </c>
+      <c r="X25" s="38">
+        <f>maint</f>
+        <v/>
+      </c>
+      <c r="Y25" s="38">
+        <f>VLOOKUP(B25,country_opex,7,FALSE)*ins_pct</f>
+        <v/>
+      </c>
+      <c r="Z25" s="38">
+        <f>charge_berth</f>
+        <v/>
+      </c>
+      <c r="AA25" s="38">
+        <f>U25+V25+W25+X25+Y25+Z25</f>
+        <v/>
+      </c>
+      <c r="AB25" s="38">
+        <f>VLOOKUP(B25,country_opex,7,FALSE)/dep_years</f>
+        <v/>
+      </c>
+      <c r="AC25" s="38">
+        <f>T25-AA25</f>
+        <v/>
+      </c>
+      <c r="AD25" s="35">
+        <f>IF(T25=0,"",AC25/T25)</f>
+        <v/>
+      </c>
+      <c r="AE25" s="36">
+        <f>IF(AC25&lt;=0,"",VLOOKUP(B25,country_opex,7,FALSE)/AC25)</f>
+        <v/>
+      </c>
+      <c r="AF25" s="33">
+        <f>((D25*O25/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D25*O25*VLOOKUP(B25,country_opex,4,FALSE))/1000</f>
+        <v/>
+      </c>
+      <c r="AG25" s="31" t="n">
+        <v>222000</v>
+      </c>
+      <c r="AH25" s="32" t="n"/>
+      <c r="AI25" s="32" t="n"/>
+      <c r="AJ25" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AK25" s="34">
+        <f>IF(AG25="","",AG25*AJ25)</f>
+        <v/>
+      </c>
+      <c r="AL25" s="34">
+        <f>IF(OR(AG25="",R25=0),"",MIN(IF(AT25="",9.9E+99,AT25),FLOOR(AK25/R25,1)))</f>
+        <v/>
+      </c>
+      <c r="AM25" s="38">
+        <f>IF(AL25="","",AL25*T25)</f>
+        <v/>
+      </c>
+      <c r="AN25" s="36">
+        <f>IF(OR(AG25="",R25=0),"",MIN(IF(AT25="",9.9E+99,AT25),AK25/R25))</f>
+        <v/>
+      </c>
+      <c r="AO25" s="38">
+        <f>IF(AN25="","",AN25*T25)</f>
+        <v/>
+      </c>
+      <c r="AP25" s="40" t="n"/>
+      <c r="AQ25" s="32" t="inlineStr">
+        <is>
+          <t>Grounded</t>
+        </is>
+      </c>
+      <c r="AR25" s="41" t="n"/>
+      <c r="AS25" s="41" t="n"/>
+      <c r="AT25" s="42" t="n"/>
+      <c r="AU25" s="43">
+        <f>IF(((S25*pax_cap*load_thin*ROUND(K25*L25*revleg_thin,0))-(((battery/range_nm)*D25*ROUND(K25*L25*revleg_thin,0)*VLOOKUP(B25,country_opex,3,FALSE))+V25+W25+X25+Y25+Z25))&lt;=0,"",VLOOKUP(B25,country_opex,7,FALSE)/((S25*pax_cap*load_thin*ROUND(K25*L25*revleg_thin,0))-(((battery/range_nm)*D25*ROUND(K25*L25*revleg_thin,0)*VLOOKUP(B25,country_opex,3,FALSE))+V25+W25+X25+Y25+Z25)))</f>
+        <v/>
+      </c>
+      <c r="AV25" s="43">
+        <f>IF(((S25*pax_cap*load_mid*ROUND(K25*L25*revleg_mid,0))-(((battery/range_nm)*D25*ROUND(K25*L25*revleg_mid,0)*VLOOKUP(B25,country_opex,3,FALSE))+V25+W25+X25+Y25+Z25))&lt;=0,"",VLOOKUP(B25,country_opex,7,FALSE)/((S25*pax_cap*load_mid*ROUND(K25*L25*revleg_mid,0))-(((battery/range_nm)*D25*ROUND(K25*L25*revleg_mid,0)*VLOOKUP(B25,country_opex,3,FALSE))+V25+W25+X25+Y25+Z25)))</f>
+        <v/>
+      </c>
+      <c r="AW25" s="43">
+        <f>IF(((S25*pax_cap*load_full*ROUND(K25*L25*revleg_full,0))-(((battery/range_nm)*D25*ROUND(K25*L25*revleg_full,0)*VLOOKUP(B25,country_opex,3,FALSE))+V25+W25+X25+Y25+Z25))&lt;=0,"",VLOOKUP(B25,country_opex,7,FALSE)/((S25*pax_cap*load_full*ROUND(K25*L25*revleg_full,0))-(((battery/range_nm)*D25*ROUND(K25*L25*revleg_full,0)*VLOOKUP(B25,country_opex,3,FALSE))+V25+W25+X25+Y25+Z25)))</f>
+        <v/>
+      </c>
+      <c r="AX25" s="44" t="n"/>
+      <c r="AY25" s="44" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="29" t="inlineStr">
+        <is>
+          <t>Yassir</t>
+        </is>
+      </c>
+      <c r="B26" s="29" t="inlineStr">
+        <is>
+          <t>Tunisia</t>
+        </is>
+      </c>
+      <c r="C26" s="30" t="inlineStr">
+        <is>
+          <t>Sfax → Sidi Youssef (Kerkennah Islands)</t>
+        </is>
+      </c>
+      <c r="D26" s="31" t="n">
+        <v>11</v>
+      </c>
+      <c r="E26" s="26" t="n"/>
+      <c r="F26" s="32" t="n"/>
+      <c r="G26" s="32" t="n"/>
+      <c r="H26" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I26" s="33">
+        <f>60*D26/cruise_kt</f>
+        <v/>
+      </c>
+      <c r="J26" s="33">
+        <f>I26+turn_min+dwell_min</f>
+        <v/>
+      </c>
+      <c r="K26" s="34">
+        <f>MIN(15,FLOOR(60*service_hr/J26,1))</f>
+        <v/>
+      </c>
+      <c r="L26" s="34">
+        <f>ROUND(365*mech_uptime*H26,0)</f>
+        <v/>
+      </c>
+      <c r="M26" s="35">
+        <f>mech_uptime</f>
+        <v/>
+      </c>
+      <c r="N26" s="35">
+        <f>revleg_sel</f>
+        <v/>
+      </c>
+      <c r="O26" s="34">
+        <f>ROUND(K26*L26*revleg_sel,0)</f>
+        <v/>
+      </c>
+      <c r="P26" s="36">
+        <f>load_sel</f>
+        <v/>
+      </c>
+      <c r="Q26" s="36">
+        <f>pax_cap*P26</f>
+        <v/>
+      </c>
+      <c r="R26" s="34">
+        <f>Q26*O26</f>
+        <v/>
+      </c>
+      <c r="S26" s="37">
+        <f>E26*discount</f>
+        <v/>
+      </c>
+      <c r="T26" s="38">
+        <f>S26*R26</f>
+        <v/>
+      </c>
+      <c r="U26" s="38">
+        <f>(battery/range_nm)*D26*O26*VLOOKUP(B26,country_opex,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="V26" s="38">
+        <f>VLOOKUP(B26,country_opex,2,FALSE)*crew_factor</f>
+        <v/>
+      </c>
+      <c r="W26" s="38">
+        <f>VLOOKUP(B26,country_opex,5,FALSE)</f>
+        <v/>
+      </c>
+      <c r="X26" s="38">
+        <f>maint</f>
+        <v/>
+      </c>
+      <c r="Y26" s="38">
+        <f>VLOOKUP(B26,country_opex,7,FALSE)*ins_pct</f>
+        <v/>
+      </c>
+      <c r="Z26" s="38">
+        <f>charge_berth</f>
+        <v/>
+      </c>
+      <c r="AA26" s="38">
+        <f>U26+V26+W26+X26+Y26+Z26</f>
+        <v/>
+      </c>
+      <c r="AB26" s="38">
+        <f>VLOOKUP(B26,country_opex,7,FALSE)/dep_years</f>
+        <v/>
+      </c>
+      <c r="AC26" s="38">
+        <f>T26-AA26</f>
+        <v/>
+      </c>
+      <c r="AD26" s="35">
+        <f>IF(T26=0,"",AC26/T26)</f>
+        <v/>
+      </c>
+      <c r="AE26" s="36">
+        <f>IF(AC26&lt;=0,"",VLOOKUP(B26,country_opex,7,FALSE)/AC26)</f>
+        <v/>
+      </c>
+      <c r="AF26" s="33">
+        <f>((D26*O26/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D26*O26*VLOOKUP(B26,country_opex,4,FALSE))/1000</f>
+        <v/>
+      </c>
+      <c r="AG26" s="31" t="n">
+        <v>1750000</v>
+      </c>
+      <c r="AH26" s="32" t="n"/>
+      <c r="AI26" s="32" t="n"/>
+      <c r="AJ26" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AK26" s="34">
+        <f>IF(AG26="","",AG26*AJ26)</f>
+        <v/>
+      </c>
+      <c r="AL26" s="34">
+        <f>IF(OR(AG26="",R26=0),"",MIN(IF(AT26="",9.9E+99,AT26),FLOOR(AK26/R26,1)))</f>
+        <v/>
+      </c>
+      <c r="AM26" s="38">
+        <f>IF(AL26="","",AL26*T26)</f>
+        <v/>
+      </c>
+      <c r="AN26" s="36">
+        <f>IF(OR(AG26="",R26=0),"",MIN(IF(AT26="",9.9E+99,AT26),AK26/R26))</f>
+        <v/>
+      </c>
+      <c r="AO26" s="38">
+        <f>IF(AN26="","",AN26*T26)</f>
+        <v/>
+      </c>
+      <c r="AP26" s="40" t="n"/>
+      <c r="AQ26" s="32" t="inlineStr">
+        <is>
+          <t>Grounded</t>
+        </is>
+      </c>
+      <c r="AR26" s="41" t="n"/>
+      <c r="AS26" s="41" t="n"/>
+      <c r="AT26" s="42" t="n"/>
+      <c r="AU26" s="43">
+        <f>IF(((S26*pax_cap*load_thin*ROUND(K26*L26*revleg_thin,0))-(((battery/range_nm)*D26*ROUND(K26*L26*revleg_thin,0)*VLOOKUP(B26,country_opex,3,FALSE))+V26+W26+X26+Y26+Z26))&lt;=0,"",VLOOKUP(B26,country_opex,7,FALSE)/((S26*pax_cap*load_thin*ROUND(K26*L26*revleg_thin,0))-(((battery/range_nm)*D26*ROUND(K26*L26*revleg_thin,0)*VLOOKUP(B26,country_opex,3,FALSE))+V26+W26+X26+Y26+Z26)))</f>
+        <v/>
+      </c>
+      <c r="AV26" s="43">
+        <f>IF(((S26*pax_cap*load_mid*ROUND(K26*L26*revleg_mid,0))-(((battery/range_nm)*D26*ROUND(K26*L26*revleg_mid,0)*VLOOKUP(B26,country_opex,3,FALSE))+V26+W26+X26+Y26+Z26))&lt;=0,"",VLOOKUP(B26,country_opex,7,FALSE)/((S26*pax_cap*load_mid*ROUND(K26*L26*revleg_mid,0))-(((battery/range_nm)*D26*ROUND(K26*L26*revleg_mid,0)*VLOOKUP(B26,country_opex,3,FALSE))+V26+W26+X26+Y26+Z26)))</f>
+        <v/>
+      </c>
+      <c r="AW26" s="43">
+        <f>IF(((S26*pax_cap*load_full*ROUND(K26*L26*revleg_full,0))-(((battery/range_nm)*D26*ROUND(K26*L26*revleg_full,0)*VLOOKUP(B26,country_opex,3,FALSE))+V26+W26+X26+Y26+Z26))&lt;=0,"",VLOOKUP(B26,country_opex,7,FALSE)/((S26*pax_cap*load_full*ROUND(K26*L26*revleg_full,0))-(((battery/range_nm)*D26*ROUND(K26*L26*revleg_full,0)*VLOOKUP(B26,country_opex,3,FALSE))+V26+W26+X26+Y26+Z26)))</f>
+        <v/>
+      </c>
+      <c r="AX26" s="44" t="n"/>
+      <c r="AY26" s="44" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="29" t="inlineStr">
+        <is>
+          <t>Yassir</t>
+        </is>
+      </c>
+      <c r="B27" s="29" t="inlineStr">
+        <is>
+          <t>Tunisia</t>
+        </is>
+      </c>
+      <c r="C27" s="30" t="inlineStr">
+        <is>
+          <t>Sousse (Port El Kantaoui) → Monastir (Marina)</t>
+        </is>
+      </c>
+      <c r="D27" s="31" t="n">
+        <v>12</v>
+      </c>
+      <c r="E27" s="26" t="n">
+        <v>32</v>
+      </c>
+      <c r="F27" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G27" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="H27" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" s="33">
+        <f>60*D27/cruise_kt</f>
+        <v/>
+      </c>
+      <c r="J27" s="33">
+        <f>I27+turn_min+dwell_min</f>
+        <v/>
+      </c>
+      <c r="K27" s="34">
+        <f>MIN(24,FLOOR(60*service_hr/J27,1))</f>
+        <v/>
+      </c>
+      <c r="L27" s="34">
+        <f>ROUND(365*mech_uptime*H27,0)</f>
+        <v/>
+      </c>
+      <c r="M27" s="35">
+        <f>mech_uptime</f>
+        <v/>
+      </c>
+      <c r="N27" s="35">
+        <f>revleg_sel</f>
+        <v/>
+      </c>
+      <c r="O27" s="34">
+        <f>ROUND(K27*L27*revleg_sel,0)</f>
+        <v/>
+      </c>
+      <c r="P27" s="36">
+        <f>load_sel</f>
+        <v/>
+      </c>
+      <c r="Q27" s="36">
+        <f>pax_cap*P27</f>
+        <v/>
+      </c>
+      <c r="R27" s="34">
+        <f>Q27*O27</f>
+        <v/>
+      </c>
+      <c r="S27" s="37">
+        <f>E27*discount</f>
+        <v/>
+      </c>
+      <c r="T27" s="38">
+        <f>S27*R27</f>
+        <v/>
+      </c>
+      <c r="U27" s="38">
+        <f>(battery/range_nm)*D27*O27*VLOOKUP(B27,country_opex,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="V27" s="38">
+        <f>VLOOKUP(B27,country_opex,2,FALSE)*crew_factor</f>
+        <v/>
+      </c>
+      <c r="W27" s="38">
+        <f>VLOOKUP(B27,country_opex,5,FALSE)</f>
+        <v/>
+      </c>
+      <c r="X27" s="38">
+        <f>maint</f>
+        <v/>
+      </c>
+      <c r="Y27" s="38">
+        <f>VLOOKUP(B27,country_opex,7,FALSE)*ins_pct</f>
+        <v/>
+      </c>
+      <c r="Z27" s="38">
+        <f>charge_berth</f>
+        <v/>
+      </c>
+      <c r="AA27" s="38">
+        <f>U27+V27+W27+X27+Y27+Z27</f>
+        <v/>
+      </c>
+      <c r="AB27" s="38">
+        <f>VLOOKUP(B27,country_opex,7,FALSE)/dep_years</f>
+        <v/>
+      </c>
+      <c r="AC27" s="38">
+        <f>T27-AA27</f>
+        <v/>
+      </c>
+      <c r="AD27" s="35">
+        <f>IF(T27=0,"",AC27/T27)</f>
+        <v/>
+      </c>
+      <c r="AE27" s="36">
+        <f>IF(AC27&lt;=0,"",VLOOKUP(B27,country_opex,7,FALSE)/AC27)</f>
+        <v/>
+      </c>
+      <c r="AF27" s="33">
+        <f>((D27*O27/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D27*O27*VLOOKUP(B27,country_opex,4,FALSE))/1000</f>
+        <v/>
+      </c>
+      <c r="AG27" s="31" t="n">
+        <v>344000</v>
+      </c>
+      <c r="AH27" s="32" t="n"/>
+      <c r="AI27" s="32" t="n"/>
+      <c r="AJ27" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AK27" s="34">
+        <f>IF(AG27="","",AG27*AJ27)</f>
+        <v/>
+      </c>
+      <c r="AL27" s="34">
+        <f>IF(OR(AG27="",R27=0),"",MIN(IF(AT27="",9.9E+99,AT27),FLOOR(AK27/R27,1)))</f>
+        <v/>
+      </c>
+      <c r="AM27" s="38">
+        <f>IF(AL27="","",AL27*T27)</f>
+        <v/>
+      </c>
+      <c r="AN27" s="36">
+        <f>IF(OR(AG27="",R27=0),"",MIN(IF(AT27="",9.9E+99,AT27),AK27/R27))</f>
+        <v/>
+      </c>
+      <c r="AO27" s="38">
+        <f>IF(AN27="","",AN27*T27)</f>
+        <v/>
+      </c>
+      <c r="AP27" s="40" t="n"/>
+      <c r="AQ27" s="32" t="inlineStr">
+        <is>
+          <t>Grounded</t>
+        </is>
+      </c>
+      <c r="AR27" s="41" t="n"/>
+      <c r="AS27" s="41" t="n"/>
+      <c r="AT27" s="42" t="n"/>
+      <c r="AU27" s="43">
+        <f>IF(((S27*pax_cap*load_thin*ROUND(K27*L27*revleg_thin,0))-(((battery/range_nm)*D27*ROUND(K27*L27*revleg_thin,0)*VLOOKUP(B27,country_opex,3,FALSE))+V27+W27+X27+Y27+Z27))&lt;=0,"",VLOOKUP(B27,country_opex,7,FALSE)/((S27*pax_cap*load_thin*ROUND(K27*L27*revleg_thin,0))-(((battery/range_nm)*D27*ROUND(K27*L27*revleg_thin,0)*VLOOKUP(B27,country_opex,3,FALSE))+V27+W27+X27+Y27+Z27)))</f>
+        <v/>
+      </c>
+      <c r="AV27" s="43">
+        <f>IF(((S27*pax_cap*load_mid*ROUND(K27*L27*revleg_mid,0))-(((battery/range_nm)*D27*ROUND(K27*L27*revleg_mid,0)*VLOOKUP(B27,country_opex,3,FALSE))+V27+W27+X27+Y27+Z27))&lt;=0,"",VLOOKUP(B27,country_opex,7,FALSE)/((S27*pax_cap*load_mid*ROUND(K27*L27*revleg_mid,0))-(((battery/range_nm)*D27*ROUND(K27*L27*revleg_mid,0)*VLOOKUP(B27,country_opex,3,FALSE))+V27+W27+X27+Y27+Z27)))</f>
+        <v/>
+      </c>
+      <c r="AW27" s="43">
+        <f>IF(((S27*pax_cap*load_full*ROUND(K27*L27*revleg_full,0))-(((battery/range_nm)*D27*ROUND(K27*L27*revleg_full,0)*VLOOKUP(B27,country_opex,3,FALSE))+V27+W27+X27+Y27+Z27))&lt;=0,"",VLOOKUP(B27,country_opex,7,FALSE)/((S27*pax_cap*load_full*ROUND(K27*L27*revleg_full,0))-(((battery/range_nm)*D27*ROUND(K27*L27*revleg_full,0)*VLOOKUP(B27,country_opex,3,FALSE))+V27+W27+X27+Y27+Z27)))</f>
+        <v/>
+      </c>
+      <c r="AX27" s="44" t="inlineStr">
         <is>
           <t>PREMIUM charter-divided tier: Port El Kantaoui per-seat catamaran / 'pirate boat' coastal cruise ~EUR 25-35 (Catamaran Amira day-cruise; half-day pirate-boat Sousse-Monastir) -&gt; midpoint ~EUR 30 x 1.08 ~= $32. This is the nearest premium per-seat water product operating on this exact coast.</t>
         </is>
       </c>
-      <c r="AY20" s="44" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="45" t="inlineStr">
-        <is>
-          <t>TOTAL / median</t>
-        </is>
-      </c>
-      <c r="T21" s="46">
-        <f>SUM(T4:T20)</f>
-        <v/>
-      </c>
-      <c r="AC21" s="46">
-        <f>SUM(AC4:AC20)</f>
-        <v/>
-      </c>
-      <c r="AD21" s="47">
-        <f>IF(T21=0,"",AC21/T21)</f>
-        <v/>
-      </c>
-      <c r="AL21" s="48">
-        <f>SUM(AL4:AL20)</f>
-        <v/>
-      </c>
-      <c r="AM21" s="46">
-        <f>SUM(AM4:AM20)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="8" t="inlineStr">
-        <is>
-          <t>Market fleet build-up — grounded floor (network-sum of raw vessel fractions per market, rounded once; subset slices excluded; legacy per-corridor-floor totals above kept for reference)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="24" t="inlineStr">
-        <is>
-          <t>Market</t>
-        </is>
-      </c>
-      <c r="B24" s="24" t="inlineStr">
-        <is>
-          <t>Fleet basis</t>
-        </is>
-      </c>
-      <c r="C24" s="24" t="inlineStr">
-        <is>
-          <t>Raw vessels (sum)</t>
-        </is>
-      </c>
-      <c r="D24" s="24" t="inlineStr">
-        <is>
-          <t>Fleet (rounded once)</t>
-        </is>
-      </c>
-      <c r="E24" s="24" t="inlineStr">
-        <is>
-          <t>Market rev/yr (raw sum)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="25" t="inlineStr">
-        <is>
-          <t>Yassir Algeria</t>
-        </is>
-      </c>
-      <c r="B25" s="13" t="inlineStr">
-        <is>
-          <t>aspirational</t>
-        </is>
-      </c>
-      <c r="C25" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D25" s="49">
-        <f>SUMIFS(AL4:AL20,A4:A20,"Yassir Algeria",AP4:AP20,"=",AQ4:AQ20,"Grounded")</f>
-        <v/>
-      </c>
-      <c r="E25" s="50">
-        <f>SUMIFS(AM4:AM20,A4:A20,"Yassir Algeria",AP4:AP20,"=",AQ4:AQ20,"Grounded")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="25" t="inlineStr">
-        <is>
-          <t>Yassir Morocco</t>
-        </is>
-      </c>
-      <c r="B26" s="13" t="inlineStr">
-        <is>
-          <t>aspirational</t>
-        </is>
-      </c>
-      <c r="C26" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D26" s="49">
-        <f>SUMIFS(AL4:AL20,A4:A20,"Yassir Morocco",AP4:AP20,"=",AQ4:AQ20,"Grounded")</f>
-        <v/>
-      </c>
-      <c r="E26" s="50">
-        <f>SUMIFS(AM4:AM20,A4:A20,"Yassir Morocco",AP4:AP20,"=",AQ4:AQ20,"Grounded")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="25" t="inlineStr">
-        <is>
-          <t>Yassir Tunisia</t>
-        </is>
-      </c>
-      <c r="B27" s="13" t="inlineStr">
-        <is>
-          <t>aspirational</t>
-        </is>
-      </c>
-      <c r="C27" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D27" s="49">
-        <f>SUMIFS(AL4:AL20,A4:A20,"Yassir Tunisia",AP4:AP20,"=",AQ4:AQ20,"Grounded")</f>
-        <v/>
-      </c>
-      <c r="E27" s="50">
-        <f>SUMIFS(AM4:AM20,A4:A20,"Yassir Tunisia",AP4:AP20,"=",AQ4:AQ20,"Grounded")</f>
-        <v/>
-      </c>
+      <c r="AY27" s="44" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="45" t="inlineStr">
         <is>
+          <t>TOTAL / median</t>
+        </is>
+      </c>
+      <c r="T28" s="46">
+        <f>SUM(T4:T27)</f>
+        <v/>
+      </c>
+      <c r="AC28" s="46">
+        <f>SUM(AC4:AC27)</f>
+        <v/>
+      </c>
+      <c r="AD28" s="47">
+        <f>IF(T28=0,"",AC28/T28)</f>
+        <v/>
+      </c>
+      <c r="AL28" s="48">
+        <f>SUM(AL4:AL27)</f>
+        <v/>
+      </c>
+      <c r="AM28" s="46">
+        <f>SUM(AM4:AM27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>Market fleet build-up — grounded floor (network-sum of raw vessel fractions per market, rounded once; subset slices excluded; legacy per-corridor-floor totals above kept for reference)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="24" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B31" s="24" t="inlineStr">
+        <is>
+          <t>Fleet basis</t>
+        </is>
+      </c>
+      <c r="C31" s="24" t="inlineStr">
+        <is>
+          <t>Raw vessels (sum)</t>
+        </is>
+      </c>
+      <c r="D31" s="24" t="inlineStr">
+        <is>
+          <t>Fleet (rounded once)</t>
+        </is>
+      </c>
+      <c r="E31" s="24" t="inlineStr">
+        <is>
+          <t>Market rev/yr (raw sum)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="25" t="inlineStr">
+        <is>
+          <t>Yassir</t>
+        </is>
+      </c>
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t>network_sum / ceil</t>
+        </is>
+      </c>
+      <c r="C32" s="23">
+        <f>SUMIFS(AN4:AN27,A4:A27,"Yassir",AP4:AP27,"=",AQ4:AQ27,"Grounded")</f>
+        <v/>
+      </c>
+      <c r="D32" s="49">
+        <f>IF(C32=0,0,CEILING(C32,1))</f>
+        <v/>
+      </c>
+      <c r="E32" s="50">
+        <f>SUMIFS(AO4:AO27,A4:A27,"Yassir",AP4:AP27,"=",AQ4:AQ27,"Grounded")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="45" t="inlineStr">
+        <is>
           <t>GROUNDED FLOOR (PUBLISHED)</t>
         </is>
       </c>
-      <c r="D28" s="48">
-        <f>SUM(D25:D27)</f>
-        <v/>
-      </c>
-      <c r="E28" s="46">
-        <f>SUM(E25:E27)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="20" t="inlineStr">
+      <c r="D33" s="48">
+        <f>SUM(D32:D32)</f>
+        <v/>
+      </c>
+      <c r="E33" s="46">
+        <f>SUM(E32:E32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="20" t="inlineStr">
         <is>
           <t>ESTIMATED DEMAND (country-median cascade; held OUT of grounded floor)</t>
         </is>
       </c>
-      <c r="D29" s="51">
-        <f>SUMIF(AQ4:AQ20,"Estimated",AL4:AL20)</f>
-        <v/>
-      </c>
-      <c r="E29" s="52">
-        <f>SUMIF(AQ4:AQ20,"Estimated",AM4:AM20)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="53" t="inlineStr">
+      <c r="D34" s="51">
+        <f>SUMIF(AQ4:AQ27,"Estimated",AL4:AL27)</f>
+        <v/>
+      </c>
+      <c r="E34" s="52">
+        <f>SUMIF(AQ4:AQ27,"Estimated",AM4:AM27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="53" t="inlineStr">
         <is>
           <t>Held for Quanta-LR (&gt;70nm, roadmap H2 2026+):</t>
         </is>
       </c>
-      <c r="C30" s="54" t="inlineStr">
+      <c r="C35" s="54" t="inlineStr">
         <is>
           <t>Tunis (La Goulette) → Palermo (Sicily, Italy) (170nm)</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="C31" s="54" t="inlineStr">
+    <row r="36">
+      <c r="C36" s="54" t="inlineStr">
         <is>
           <t>Nador (Beni Ensar) → Almeria (Spain) (92nm)</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="C32" s="54" t="inlineStr">
+    <row r="37">
+      <c r="C37" s="54" t="inlineStr">
         <is>
           <t>Port d'Oran → Mostaganem port (81.7nm)</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="C33" s="54" t="inlineStr">
+    <row r="38">
+      <c r="C38" s="54" t="inlineStr">
         <is>
           <t>Port de Béjaïa → Port d'Alger (113.8nm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="C39" s="54" t="inlineStr">
+        <is>
+          <t>Dakar → Saint-Louis (du Senegal) (90nm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="C40" s="54" t="inlineStr">
+        <is>
+          <t>Dakar (Gare maritime / Port) → Ziguinchor (Port de Ziguinchor, Casamance) (200nm)</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A30:L30"/>
     <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A23:L23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5703,7 +6911,7 @@
         </is>
       </c>
       <c r="C11" s="39" t="n">
-        <v>0.0922</v>
+        <v>0.0929</v>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>

</xml_diff>